<commit_message>
completed results of APD and prepartion of APD+ Terr
</commit_message>
<xml_diff>
--- a/src/data/output/apd_output.xlsx
+++ b/src/data/output/apd_output.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,11 @@
       <name val="Calibri"/>
       <color rgb="FF2C3E50"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -51,13 +56,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -529,25 +537,25 @@
           <t>TS-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>0097567</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>42668.00</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>1680.00</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>1280.04</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="3" t="n">
         <v>45628.04</v>
       </c>
     </row>
@@ -557,25 +565,25 @@
           <t>TS-002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>0097602</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>16078.00</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>620.00</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>759.76</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="3" t="n">
         <v>17457.76</v>
       </c>
     </row>
@@ -585,25 +593,25 @@
           <t>TS-003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>0097624</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>4573.00</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>365.00</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>224.68</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
         <v>5162.68</v>
       </c>
     </row>
@@ -613,25 +621,25 @@
           <t>TS-004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>0097646</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>10475.00</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>585.00</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>314.25</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="3" t="n">
         <v>11374.25</v>
       </c>
     </row>
@@ -641,25 +649,25 @@
           <t>TS-005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>0097651</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>13189.00</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>775.00</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="3" t="n">
         <v>314.19</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="3" t="n">
         <v>14283.08</v>
       </c>
     </row>
@@ -669,30 +677,26 @@
           <t>TS-006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>0097665</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>5317.00</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>435.00</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>129.42</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>5883.43</t>
-        </is>
+      <c r="E7" s="3" t="n">
+        <v>129.42</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>5883.43</v>
       </c>
     </row>
     <row r="8">
@@ -701,30 +705,26 @@
           <t>TS-007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>0097679</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>26594.00</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1519.78</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D8" s="3" t="n">
+        <v>1519.78</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>1329.70</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>29443.48</t>
-        </is>
+      <c r="F8" s="3" t="n">
+        <v>29443.48</v>
       </c>
     </row>
     <row r="9">
@@ -733,27 +733,27 @@
           <t>TS-008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>0097683</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>14810.00</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>1190.00</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>320.00</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>16320.00</t>
         </is>
@@ -765,30 +765,26 @@
           <t>TS-009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>0097684</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>10783.00</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>430.00</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>510.19</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>11723.19</t>
-        </is>
+      <c r="E10" s="3" t="n">
+        <v>510.19</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>11723.19</v>
       </c>
     </row>
     <row r="11">
@@ -797,30 +793,26 @@
           <t>TS-010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>0097693</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>9135.00</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>825.00</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>453.18</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>10413.18</t>
-        </is>
+      <c r="E11" s="3" t="n">
+        <v>453.18</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>10413.18</v>
       </c>
     </row>
     <row r="12">
@@ -829,6 +821,27 @@
           <t>TS-011</t>
         </is>
       </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>0097955</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>4783.00</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>370.00</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>115.94</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>5270.74</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -836,6 +849,27 @@
           <t>TS-012</t>
         </is>
       </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>0097957</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>3371.00</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>210.00</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>71.62</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>3652.62</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -843,6 +877,25 @@
           <t>TS-013</t>
         </is>
       </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>0098000</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>5857.00</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>472.57</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>292.85</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>6622.42</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -850,6 +903,27 @@
           <t>TS-014</t>
         </is>
       </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>0098001</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>4956.00</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>645.00</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>148.68</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>5749.68</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -857,6 +931,27 @@
           <t>TS-015</t>
         </is>
       </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>0097972</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>4423.00</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>140.00</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>91.26000000000001</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>4654.26</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -864,6 +959,27 @@
           <t>TS-016</t>
         </is>
       </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>0097973</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>7350.00</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>535.00</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>358.77</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>8243.77</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -871,6 +987,27 @@
           <t>TS-017</t>
         </is>
       </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>0097978</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>5384.00</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>330.00</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>161.52</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>5875.52</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -878,6 +1015,27 @@
           <t>TS-018</t>
         </is>
       </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>0098095</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>4435.00</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>515.00</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>225.23</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>5175.23</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -885,6 +1043,27 @@
           <t>TS-019</t>
         </is>
       </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>0098125</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>3155.00</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>230.00</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>94.65000000000001</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>3479.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -892,6 +1071,25 @@
           <t>TS-020</t>
         </is>
       </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>0098102</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>5863.00</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>557.59</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>293.15</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>6713.74</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -899,6 +1097,25 @@
           <t>TS-021</t>
         </is>
       </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>0098096</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>3927.00</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>256.78</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>196.35</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>4380.13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -906,6 +1123,25 @@
           <t>TS-022</t>
         </is>
       </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>0098099</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>6445.00</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>489.34</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>322.25</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>7256.59</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -913,6 +1149,27 @@
           <t>TS-023</t>
         </is>
       </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>0097981</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>8421.00</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>170.00</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>252.63</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>8843.629999999999</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -920,6 +1177,27 @@
           <t>TS-024</t>
         </is>
       </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>0098097</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>3648.00</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>345.94</v>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>182.40</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>4176.34</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -927,6 +1205,27 @@
           <t>TS-025</t>
         </is>
       </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>0098100</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>4833.00</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>325.00</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>234.69</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>5392.69</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -934,6 +1233,31 @@
           <t>TS-026</t>
         </is>
       </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>0098098</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>6200.00</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>543.60</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>310.00</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>7053.60</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -941,6 +1265,27 @@
           <t>TS-027</t>
         </is>
       </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>0097989</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>6417.00</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>235.00</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>192.51</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>6844.51</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -948,6 +1293,27 @@
           <t>TS-028</t>
         </is>
       </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>0098101</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>2495.00</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>215.00</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>123.31</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>2833.31</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -955,6 +1321,27 @@
           <t>TS-029</t>
         </is>
       </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>0098106</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>5745.00</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>620.00</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>190.95</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>6555.95</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -962,6 +1349,27 @@
           <t>TS-030</t>
         </is>
       </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>0098103</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>3575.00</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>225.00</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>107.25</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>3907.25</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -969,6 +1377,27 @@
           <t>TS-031</t>
         </is>
       </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>0097985</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>7903.00</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>830.00</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>261.99</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>8994.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -976,6 +1405,31 @@
           <t>TS-032</t>
         </is>
       </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>0097995</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>6865.00</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>140.00</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>140.10</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>7145.10</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -983,6 +1437,27 @@
           <t>TS-033</t>
         </is>
       </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>0097999</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>4026.00</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>442.08</v>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>201.30</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>4669.38</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -990,6 +1465,27 @@
           <t>TS-034</t>
         </is>
       </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>0097997</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>5377.00</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>330.00</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>114.14</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>5821.14</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -997,6 +1493,27 @@
           <t>TS-035</t>
         </is>
       </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>0097992</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>4376.00</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>348.13</v>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>218.80</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>4942.93</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1004,6 +1521,27 @@
           <t>TS-036</t>
         </is>
       </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>0097996</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>3211.00</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>455.00</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>96.33</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>3762.33</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1011,6 +1549,27 @@
           <t>TS-037</t>
         </is>
       </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>0097994</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>4973.00</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>205.00</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>155.34</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>5333.34</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1018,6 +1577,27 @@
           <t>TS-038</t>
         </is>
       </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>0097998</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>2482.00</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>290.00</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>74.45999999999999</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>2846.46</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1025,6 +1605,27 @@
           <t>TS-039</t>
         </is>
       </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>0097993</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>3542.00</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>350.00</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>116.76</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>4008.76</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1032,6 +1633,27 @@
           <t>TS-040</t>
         </is>
       </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>0097991</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>2862.00</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>475.00</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>85.86</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>3422.86</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1039,6 +1661,27 @@
           <t>TS-041</t>
         </is>
       </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>0098105</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>5217.00</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>435.00</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>113.04</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>5765.04</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1046,6 +1689,27 @@
           <t>TS-042</t>
         </is>
       </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>0098104</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>2282.00</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>280.00</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>57.65</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>2620.55</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1053,6 +1717,27 @@
           <t>TS-043</t>
         </is>
       </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>0098006</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>7938.00</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>475.00</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>252.39</v>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>8665.389999999999</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1060,6 +1745,27 @@
           <t>TS-044</t>
         </is>
       </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>0098011</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>3972.00</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>425.00</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>119.16</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>4516.16</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1067,6 +1773,27 @@
           <t>TS-045</t>
         </is>
       </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>0098004</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>2142.00</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>190.00</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>64.26000000000001</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>2396.26</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1074,6 +1801,27 @@
           <t>TS-046</t>
         </is>
       </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>0098107</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>4692.00</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>530.00</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>156.66</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>5378.66</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1081,6 +1829,27 @@
           <t>TS-047</t>
         </is>
       </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>0098136</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>6332.00</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>370.00</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>304.94</v>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>7006.94</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1088,6 +1857,27 @@
           <t>TS-048</t>
         </is>
       </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>0098110</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>6364.00</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>745.00</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>190.92</v>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>7299.92</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1095,6 +1885,27 @@
           <t>TS-049</t>
         </is>
       </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>0098013</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>3213.00</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>210.00</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>155.75</v>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>3578.75</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1102,6 +1913,27 @@
           <t>TS-050</t>
         </is>
       </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>0098014</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>9477.00</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>663.39</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>284.31</v>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>10424.70</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1109,6 +1941,25 @@
           <t>TS-051</t>
         </is>
       </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>0098012</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>4353.00</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>153.06</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>217.65</v>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>4723.71</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1116,6 +1967,27 @@
           <t>TS-052</t>
         </is>
       </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>0098015</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>2506.00</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>365.00</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>86.13</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>2957.13</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1123,6 +1995,27 @@
           <t>TS-053</t>
         </is>
       </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>0098018</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>4858.00</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>339.57</v>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>242.90</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>5440.47</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1130,6 +2023,29 @@
           <t>TS-054</t>
         </is>
       </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>0098016</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>2572.00</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>330.00</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>65.30</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>2968.32</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1137,6 +2053,27 @@
           <t>TS-055</t>
         </is>
       </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>0098017</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>2546.00</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>387.64</v>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>127.30</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>3060.94</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1144,6 +2081,27 @@
           <t>TS-056</t>
         </is>
       </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>0098019</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>7237.00</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>275.00</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>150.24</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>7662.24</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1151,6 +2109,27 @@
           <t>TS-057</t>
         </is>
       </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>0098022</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>5377.00</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>465.00</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>265.81</v>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>6107.81</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1158,6 +2137,27 @@
           <t>TS-058</t>
         </is>
       </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>0098021</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>3824.00</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>526.47</v>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>191.20</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>4541.67</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1165,6 +2165,27 @@
           <t>TS-059</t>
         </is>
       </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>0098020</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>4992.00</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>169.98</v>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>249.60</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>5411.58</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1172,6 +2193,27 @@
           <t>TS-060</t>
         </is>
       </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>0098023</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>3489.00</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>260.00</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>104.67</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>3853.67</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1179,6 +2221,27 @@
           <t>TS-061</t>
         </is>
       </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>0098024</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>8185.00</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>320.00</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>386.98</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>8891.98</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1186,6 +2249,27 @@
           <t>TS-062</t>
         </is>
       </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>0098029</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>3970.00</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>336.91</v>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>198.50</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>4505.41</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1193,6 +2277,27 @@
           <t>TS-063</t>
         </is>
       </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>0098025</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>3993.00</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>190.00</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>190.33</v>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>4373.33</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1200,6 +2305,27 @@
           <t>TS-064</t>
         </is>
       </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>0098028</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>5999.00</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>515.00</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>296.39</v>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>6810.39</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1207,6 +2333,27 @@
           <t>TS-065</t>
         </is>
       </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>0098026</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>4452.00</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>500.00</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>133.56</v>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>5085.56</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1214,6 +2361,27 @@
           <t>TS-066</t>
         </is>
       </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>0098031</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>5918.00</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>365.00</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>141.37</v>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>6426.57</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1221,6 +2389,25 @@
           <t>TS-067</t>
         </is>
       </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>0098027</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>3587.00</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>185.76</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>179.35</v>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>3952.11</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1228,6 +2415,27 @@
           <t>TS-068</t>
         </is>
       </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>0098030</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>5536.00</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>685.00</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>166.08</v>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>6387.08</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1235,6 +2443,25 @@
           <t>TS-069</t>
         </is>
       </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>0098032</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>2757.00</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>333.27</v>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>137.85</v>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>3228.12</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -1242,6 +2469,27 @@
           <t>TS-070</t>
         </is>
       </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>0098033</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>6119.00</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>275.00</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>191.82</v>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>6585.82</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -1249,6 +2497,27 @@
           <t>TS-071</t>
         </is>
       </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>0098034</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>3598.00</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>405.00</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>182.14</v>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>4185.14</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -1256,6 +2525,27 @@
           <t>TS-072</t>
         </is>
       </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>0098035</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>3186.00</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>489.56</v>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>159.30</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>3834.86</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -1263,6 +2553,31 @@
           <t>TS-073</t>
         </is>
       </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>0098036</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>5460.00</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>250.00</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>171.30</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>5881.30</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -1270,6 +2585,27 @@
           <t>TS-074</t>
         </is>
       </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>0098037</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>4548.00</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>275.00</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>108.52</v>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>4933.21</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -1277,6 +2613,27 @@
           <t>TS-075</t>
         </is>
       </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>0098038</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>5268.00</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>595.00</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>175.89</v>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>6038.89</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -1284,6 +2641,27 @@
           <t>TS-076</t>
         </is>
       </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>0098039</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>2676.00</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>185.00</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>85.83</v>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>2946.83</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -1291,6 +2669,29 @@
           <t>TS-077</t>
         </is>
       </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>0098040</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>6180.00</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>555.00</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>151.54</v>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>6888.90</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -1298,6 +2699,27 @@
           <t>TS-078</t>
         </is>
       </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>0098137</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>4990.00</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>125.78</v>
+      </c>
+      <c r="F79" s="3" t="n">
+        <v>5717.74</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -1305,6 +2727,27 @@
           <t>TS-079</t>
         </is>
       </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>0098042</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>5494.00</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>275.00</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="n">
+        <v>164.82</v>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>5933.82</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -1312,6 +2755,31 @@
           <t>TS-080</t>
         </is>
       </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>0098139</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>5839.00</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>395.00</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>140.27</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>6376.45</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -1319,6 +2787,31 @@
           <t>TS-081</t>
         </is>
       </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>0098140</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>3047.00</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>320.00</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>101.01</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>3468.01</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -1326,6 +2819,27 @@
           <t>TS-082</t>
         </is>
       </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>0098052</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>2349.00</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>215.00</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>57.69</v>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>2622.59</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -1333,6 +2847,27 @@
           <t>TS-083</t>
         </is>
       </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>0098044</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>3841.00</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>345.00</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>125.58</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>4311.58</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -1340,6 +2875,31 @@
           <t>TS-084</t>
         </is>
       </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>0098050</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>5995.00</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>365.00</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>190.80</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>6550.80</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -1347,6 +2907,27 @@
           <t>TS-085</t>
         </is>
       </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>0098047</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>3532.00</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>355.00</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>105.96</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>3992.96</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -1354,6 +2935,27 @@
           <t>TS-086</t>
         </is>
       </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>0098051</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>6935.00</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>415.00</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="n">
+        <v>165.38</v>
+      </c>
+      <c r="F87" s="3" t="n">
+        <v>7517.95</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1361,6 +2963,27 @@
           <t>TS-087</t>
         </is>
       </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>0098045</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>5297.00</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>435.00</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>260.81</v>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>5992.81</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -1368,6 +2991,27 @@
           <t>TS-088</t>
         </is>
       </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>0098049</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>2616.00</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>312.85</v>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>130.80</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>3059.65</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -1375,6 +3019,27 @@
           <t>TS-089</t>
         </is>
       </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>0098058</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>4930.00</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>425.00</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="n">
+        <v>120.49</v>
+      </c>
+      <c r="F90" s="3" t="n">
+        <v>5477.36</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -1382,6 +3047,27 @@
           <t>TS-090</t>
         </is>
       </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>0098062</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>3702.00</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>450.00</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="n">
+        <v>111.06</v>
+      </c>
+      <c r="F91" s="3" t="n">
+        <v>4263.06</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -1389,6 +3075,27 @@
           <t>TS-091</t>
         </is>
       </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>0098071</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>5377.00</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>305.00</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="n">
+        <v>161.31</v>
+      </c>
+      <c r="F92" s="3" t="n">
+        <v>5843.31</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1396,6 +3103,27 @@
           <t>TS-092</t>
         </is>
       </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>0098057</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>3346.00</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>430.00</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="n">
+        <v>113.28</v>
+      </c>
+      <c r="F93" s="3" t="n">
+        <v>3889.28</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -1403,6 +3131,27 @@
           <t>TS-093</t>
         </is>
       </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>0098061</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>3320.00</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>325.00</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="n">
+        <v>109.35</v>
+      </c>
+      <c r="F94" s="3" t="n">
+        <v>3754.35</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -1410,6 +3159,27 @@
           <t>TS-094</t>
         </is>
       </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>0098059</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>3262.00</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>210.00</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="n">
+        <v>69.44</v>
+      </c>
+      <c r="F95" s="3" t="n">
+        <v>3541.44</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1417,6 +3187,27 @@
           <t>TS-095</t>
         </is>
       </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>0098064</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>5708.00</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>450.00</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="n">
+        <v>280.19</v>
+      </c>
+      <c r="F96" s="3" t="n">
+        <v>6438.19</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1424,6 +3215,27 @@
           <t>TS-096</t>
         </is>
       </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>0098060</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>3488.00</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>505.00</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="n">
+        <v>119.79</v>
+      </c>
+      <c r="F97" s="3" t="n">
+        <v>4112.79</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1431,6 +3243,27 @@
           <t>TS-097</t>
         </is>
       </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>0098063</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>3358.00</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>160.00</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="n">
+        <v>100.74</v>
+      </c>
+      <c r="F98" s="3" t="n">
+        <v>3618.74</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -1438,6 +3271,31 @@
           <t>TS-098</t>
         </is>
       </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>0098069</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>6340.00</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>500.00</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>190.20</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>7030.20</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -1445,6 +3303,27 @@
           <t>TS-099</t>
         </is>
       </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>0098070</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>6892.00</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>345.00</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="n">
+        <v>162.83</v>
+      </c>
+      <c r="F100" s="3" t="n">
+        <v>7402.36</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -1452,6 +3331,25 @@
           <t>TS-100</t>
         </is>
       </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>0098073</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>6107.00</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="n">
+        <v>693.3200000000001</v>
+      </c>
+      <c r="E101" s="3" t="n">
+        <v>305.35</v>
+      </c>
+      <c r="F101" s="3" t="n">
+        <v>7105.67</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -1459,6 +3357,27 @@
           <t>TS-101</t>
         </is>
       </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>0098075</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>4006.00</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>225.00</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="n">
+        <v>120.18</v>
+      </c>
+      <c r="F102" s="3" t="n">
+        <v>4351.18</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -1466,6 +3385,27 @@
           <t>TS-102</t>
         </is>
       </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>0098074</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>4463.00</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>430.00</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="n">
+        <v>146.79</v>
+      </c>
+      <c r="F103" s="3" t="n">
+        <v>5039.79</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -1473,6 +3413,27 @@
           <t>TS-103</t>
         </is>
       </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>0098076</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>5377.00</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>325.00</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="n">
+        <v>161.31</v>
+      </c>
+      <c r="F104" s="3" t="n">
+        <v>5863.31</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -1480,6 +3441,27 @@
           <t>TS-104</t>
         </is>
       </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>0098077</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>3453.00</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>330.00</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="n">
+        <v>85.12</v>
+      </c>
+      <c r="F105" s="3" t="n">
+        <v>3869.44</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -1487,6 +3469,27 @@
           <t>TS-105</t>
         </is>
       </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>0098078</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>2866.00</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>185.00</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="n">
+        <v>68.65000000000001</v>
+      </c>
+      <c r="F106" s="3" t="n">
+        <v>3120.72</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -1494,6 +3497,27 @@
           <t>TS-106</t>
         </is>
       </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>0098079</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>6521.00</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>475.00</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="n">
+        <v>195.63</v>
+      </c>
+      <c r="F107" s="3" t="n">
+        <v>7191.63</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -1501,6 +3525,27 @@
           <t>TS-107</t>
         </is>
       </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>0098080</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>3927.00</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>305.00</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="n">
+        <v>192.56</v>
+      </c>
+      <c r="F108" s="3" t="n">
+        <v>4424.56</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -1508,6 +3553,27 @@
           <t>TS-108</t>
         </is>
       </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>0098081</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>4759.00</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>440.00</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="n">
+        <v>142.77</v>
+      </c>
+      <c r="F109" s="3" t="n">
+        <v>5341.77</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -1515,6 +3581,27 @@
           <t>TS-109</t>
         </is>
       </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>0098082</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>3199.00</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>215.00</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="n">
+        <v>95.97</v>
+      </c>
+      <c r="F110" s="3" t="n">
+        <v>3509.97</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -1522,6 +3609,27 @@
           <t>TS-110</t>
         </is>
       </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>0098083</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>3714.00</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>285.00</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="n">
+        <v>111.42</v>
+      </c>
+      <c r="F111" s="3" t="n">
+        <v>4110.42</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -1529,6 +3637,27 @@
           <t>TS-111</t>
         </is>
       </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>0098085</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>8001.00</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>780.00</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="n">
+        <v>240.03</v>
+      </c>
+      <c r="F112" s="3" t="n">
+        <v>9021.030000000001</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -1536,6 +3665,27 @@
           <t>TS-112</t>
         </is>
       </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>0098084</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>4440.00</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="n">
+        <v>238.32</v>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>222.00</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="n">
+        <v>4900.32</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -1543,6 +3693,29 @@
           <t>TS-113</t>
         </is>
       </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>0098088</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>5244.00</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>645.00</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>132.50</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="n">
+        <v>6023.56</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -1550,6 +3723,27 @@
           <t>TS-114</t>
         </is>
       </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>0098086</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>6907.00</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>140.00</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="n">
+        <v>211.41</v>
+      </c>
+      <c r="F115" s="3" t="n">
+        <v>7258.41</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -1557,6 +3751,31 @@
           <t>TS-115</t>
         </is>
       </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>0098089</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>8565.00</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>705.00</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>278.10</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>9548.10</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -1564,6 +3783,27 @@
           <t>TS-116</t>
         </is>
       </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>0098090</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>5216.00</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="n">
+        <v>345.65</v>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>260.80</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="n">
+        <v>5822.45</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -1571,6 +3811,31 @@
           <t>TS-117</t>
         </is>
       </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>0098138</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>4612.00</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>345.00</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>225.54</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>5182.54</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -1578,6 +3843,31 @@
           <t>TS-118</t>
         </is>
       </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>0098141</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>4683.00</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>500.00</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>140.49</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>5323.49</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -1585,11 +3875,61 @@
           <t>TS-119</t>
         </is>
       </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>0098143</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>8571.00</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>255.00</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>257.13</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>9083.13</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
           <t>TS-120</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>0098142</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>4459.00</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>430.00</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>97.78</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>4986.78</t>
         </is>
       </c>
     </row>

</xml_diff>